<commit_message>
Ajustes esteticos finales: formato de fecha, separacion de NIT y DV, llenado de CDP/RPC/Ciudad y nombre corto en archivos ZIP
</commit_message>
<xml_diff>
--- a/doc/2. DS-4121-0411 Cuota 6 -YESID PIEDRAHITA.xlsx
+++ b/doc/2. DS-4121-0411 Cuota 6 -YESID PIEDRAHITA.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\Documento cuenta\Informe de actividades\2026\CUOTA 6\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC889C0-5A23-43B8-9D20-9541CD13061B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Documento Equivalente" sheetId="1" r:id="rId1"/>
@@ -148,13 +142,13 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="5">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;\ * #,##0.00_);_(&quot;$&quot;\ * \(#,##0.00\);_(&quot;$&quot;\ * &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
-    <numFmt numFmtId="165" formatCode="##,###"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;\ * #,##0.00_);_(&quot;$&quot;\ * \(#,##0.00\);_(&quot;$&quot;\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="167" formatCode="##,###"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -206,7 +200,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -229,6 +223,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD8D8D8"/>
         <bgColor rgb="FFD8D8D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -726,7 +726,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -744,16 +744,13 @@
     <xf numFmtId="1" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="12" fontId="6" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -762,33 +759,110 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="12" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -798,90 +872,20 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -914,7 +918,7 @@
         <xdr:cNvPr id="3" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -969,7 +973,7 @@
         <xdr:cNvPr id="4" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1024,7 +1028,7 @@
         <xdr:cNvPr id="2" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1079,7 +1083,7 @@
         <xdr:cNvPr id="5" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1134,7 +1138,7 @@
         <xdr:cNvPr id="6" name="Shape 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1235,7 +1239,7 @@
         <xdr:cNvPr id="7" name="Shape 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000007000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1254,7 +1258,7 @@
           <xdr:cNvPr id="8" name="Shape 6">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000008000000}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1273,7 +1277,7 @@
             <xdr:cNvPr id="9" name="Shape 7">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000009000000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1316,7 +1320,7 @@
             <xdr:cNvPr id="10" name="Shape 8">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000A000000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1335,7 +1339,7 @@
               <xdr:cNvPr id="11" name="Shape 9">
                 <a:extLst>
                   <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000B000000}"/>
                   </a:ext>
                 </a:extLst>
               </xdr:cNvPr>
@@ -1380,7 +1384,7 @@
               <xdr:cNvPr id="12" name="Shape 10">
                 <a:extLst>
                   <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000C000000}"/>
                   </a:ext>
                 </a:extLst>
               </xdr:cNvPr>
@@ -1399,7 +1403,7 @@
                 <xdr:cNvPr id="13" name="Shape 11">
                   <a:extLst>
                     <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000D000000}"/>
                     </a:ext>
                   </a:extLst>
                 </xdr:cNvPr>
@@ -1444,7 +1448,7 @@
                 <xdr:cNvPr id="14" name="Shape 12">
                   <a:extLst>
                     <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
+                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000E000000}"/>
                     </a:ext>
                   </a:extLst>
                 </xdr:cNvPr>
@@ -1463,7 +1467,7 @@
                   <xdr:cNvPr id="15" name="Shape 13">
                     <a:extLst>
                       <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
+                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000F000000}"/>
                       </a:ext>
                     </a:extLst>
                   </xdr:cNvPr>
@@ -1508,7 +1512,7 @@
                   <xdr:cNvPr id="16" name="Shape 14">
                     <a:extLst>
                       <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
+                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000010000000}"/>
                       </a:ext>
                     </a:extLst>
                   </xdr:cNvPr>
@@ -1527,7 +1531,7 @@
                     <xdr:cNvPr id="17" name="Shape 15">
                       <a:extLst>
                         <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
+                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000011000000}"/>
                         </a:ext>
                       </a:extLst>
                     </xdr:cNvPr>
@@ -1572,7 +1576,7 @@
                     <xdr:cNvPr id="18" name="Shape 16">
                       <a:extLst>
                         <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
+                          <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000012000000}"/>
                         </a:ext>
                       </a:extLst>
                     </xdr:cNvPr>
@@ -1591,7 +1595,7 @@
                       <xdr:cNvPr id="19" name="Shape 17">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
+                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000013000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1636,7 +1640,7 @@
                       <xdr:cNvPr id="20" name="Shape 18">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
+                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000014000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -1655,7 +1659,7 @@
                         <xdr:cNvPr id="21" name="Shape 19">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000015000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1706,7 +1710,7 @@
                         <xdr:cNvPr id="22" name="Shape 20">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000016000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1782,7 +1786,7 @@
                         <xdr:cNvPr id="23" name="Shape 21">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000017000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1850,7 +1854,7 @@
                         <xdr:cNvPr id="24" name="Shape 22">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000018000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -1918,7 +1922,7 @@
                         <xdr:cNvPr id="25" name="Shape 23">
                           <a:extLst>
                             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
+                              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000019000000}"/>
                             </a:ext>
                           </a:extLst>
                         </xdr:cNvPr>
@@ -2093,7 +2097,7 @@
                       <xdr:cNvPr id="26" name="Shape 24" descr="escudo">
                         <a:extLst>
                           <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
+                            <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00001A000000}"/>
                           </a:ext>
                         </a:extLst>
                       </xdr:cNvPr>
@@ -2329,7 +2333,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -2347,15 +2351,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A1" s="64"/>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
+      <c r="A1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -2375,15 +2379,15 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A2" s="51"/>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
@@ -2403,15 +2407,15 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A3" s="51"/>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
+      <c r="A3" s="23"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -2431,15 +2435,15 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="15" customHeight="1">
-      <c r="A4" s="51"/>
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
-      <c r="F4" s="51"/>
-      <c r="G4" s="51"/>
-      <c r="H4" s="51"/>
-      <c r="I4" s="51"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -2459,15 +2463,15 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="16.5" customHeight="1">
-      <c r="A5" s="51"/>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
-      <c r="H5" s="51"/>
-      <c r="I5" s="51"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -2487,15 +2491,15 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" s="51"/>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -2515,15 +2519,15 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A7" s="51"/>
-      <c r="B7" s="51"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
-      <c r="G7" s="51"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="51"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -2543,15 +2547,15 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A8" s="51"/>
-      <c r="B8" s="51"/>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
-      <c r="F8" s="51"/>
-      <c r="G8" s="51"/>
-      <c r="H8" s="51"/>
-      <c r="I8" s="51"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -2571,15 +2575,15 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="13.5" customHeight="1">
-      <c r="A9" s="51"/>
-      <c r="B9" s="51"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
-      <c r="I9" s="51"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -2599,15 +2603,15 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1">
-      <c r="A10" s="51"/>
-      <c r="B10" s="51"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51"/>
-      <c r="G10" s="51"/>
-      <c r="H10" s="51"/>
-      <c r="I10" s="51"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -2627,17 +2631,17 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A11" s="57" t="s">
+      <c r="A11" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="58"/>
-      <c r="C11" s="58"/>
-      <c r="D11" s="58"/>
-      <c r="E11" s="58"/>
-      <c r="F11" s="58"/>
-      <c r="G11" s="58"/>
-      <c r="H11" s="58"/>
-      <c r="I11" s="59"/>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="26"/>
       <c r="J11" s="2">
         <v>1</v>
       </c>
@@ -2659,15 +2663,15 @@
       <c r="Z11" s="3"/>
     </row>
     <row r="12" spans="1:26" ht="39.75" customHeight="1">
-      <c r="A12" s="65" t="s">
+      <c r="A12" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="66"/>
-      <c r="C12" s="67"/>
-      <c r="D12" s="68">
+      <c r="B12" s="28"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="65">
         <v>46197</v>
       </c>
-      <c r="E12" s="31"/>
+      <c r="E12" s="66"/>
       <c r="F12" s="4" t="s">
         <v>2</v>
       </c>
@@ -2677,10 +2681,10 @@
       <c r="H12" s="6">
         <v>4121</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="67" t="s">
         <v>37</v>
       </c>
-      <c r="J12" s="8"/>
+      <c r="J12" s="7"/>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
@@ -2699,26 +2703,26 @@
       <c r="Z12" s="3"/>
     </row>
     <row r="13" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A13" s="55" t="s">
+      <c r="A13" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="53" t="s">
+      <c r="B13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="9" t="s">
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="9">
         <v>890399011</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="10">
         <v>3</v>
       </c>
-      <c r="J13" s="8"/>
+      <c r="J13" s="7"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
@@ -2737,24 +2741,24 @@
       <c r="Z13" s="3"/>
     </row>
     <row r="14" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A14" s="55" t="s">
+      <c r="A14" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="35"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="54" t="s">
+      <c r="B14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="35"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="12" t="s">
+      <c r="E14" s="18"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="H14" s="56">
+      <c r="H14" s="20">
         <v>4121</v>
       </c>
-      <c r="I14" s="40"/>
-      <c r="J14" s="8"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="7"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
@@ -2773,24 +2777,24 @@
       <c r="Z14" s="3"/>
     </row>
     <row r="15" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A15" s="55" t="s">
+      <c r="A15" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="35"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="41" t="s">
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="35"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="12" t="s">
+      <c r="E15" s="18"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="56">
+      <c r="H15" s="20">
         <v>8896744</v>
       </c>
-      <c r="I15" s="40"/>
-      <c r="J15" s="8"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="7"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
@@ -2809,17 +2813,17 @@
       <c r="Z15" s="3"/>
     </row>
     <row r="16" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A16" s="57" t="s">
+      <c r="A16" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="58"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="58"/>
-      <c r="F16" s="58"/>
-      <c r="G16" s="58"/>
-      <c r="H16" s="58"/>
-      <c r="I16" s="59"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="26"/>
       <c r="J16" s="2">
         <v>2</v>
       </c>
@@ -2841,29 +2845,29 @@
       <c r="Z16" s="3"/>
     </row>
     <row r="17" spans="1:26" ht="45" customHeight="1">
-      <c r="A17" s="60" t="s">
+      <c r="A17" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="61"/>
-      <c r="C17" s="62"/>
-      <c r="D17" s="63" t="s">
+      <c r="B17" s="35"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="61"/>
-      <c r="F17" s="62"/>
-      <c r="G17" s="13" t="s">
+      <c r="E17" s="35"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H17" s="14">
+      <c r="H17" s="13">
         <v>16839817</v>
       </c>
-      <c r="I17" s="15">
+      <c r="I17" s="14">
         <v>0</v>
       </c>
-      <c r="J17" s="8"/>
+      <c r="J17" s="7"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
-      <c r="M17" s="16"/>
+      <c r="M17" s="15"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
@@ -2879,27 +2883,27 @@
       <c r="Z17" s="3"/>
     </row>
     <row r="18" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A18" s="55" t="s">
+      <c r="A18" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="35"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="53" t="s">
+      <c r="B18" s="18"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="E18" s="35"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="12" t="s">
+      <c r="E18" s="18"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="H18" s="54" t="s">
+      <c r="H18" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="40"/>
-      <c r="J18" s="8"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="7"/>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
-      <c r="M18" s="16"/>
+      <c r="M18" s="15"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
@@ -2915,27 +2919,27 @@
       <c r="Z18" s="3"/>
     </row>
     <row r="19" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="57" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21" t="s">
+      <c r="B19" s="41"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="19"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="12" t="s">
+      <c r="E19" s="41"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="H19" s="22">
+      <c r="H19" s="59">
         <v>3016744172</v>
       </c>
-      <c r="I19" s="23"/>
-      <c r="J19" s="8"/>
+      <c r="I19" s="42"/>
+      <c r="J19" s="7"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
-      <c r="M19" s="16"/>
+      <c r="M19" s="15"/>
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
@@ -2951,17 +2955,17 @@
       <c r="Z19" s="3"/>
     </row>
     <row r="20" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="26"/>
+      <c r="B20" s="61"/>
+      <c r="C20" s="61"/>
+      <c r="D20" s="61"/>
+      <c r="E20" s="61"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="61"/>
+      <c r="H20" s="61"/>
+      <c r="I20" s="62"/>
       <c r="J20" s="2">
         <v>3</v>
       </c>
@@ -2983,19 +2987,19 @@
       <c r="Z20" s="3"/>
     </row>
     <row r="21" spans="1:26" ht="24.75" customHeight="1">
-      <c r="A21" s="27" t="s">
+      <c r="A21" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="32" t="s">
+      <c r="B21" s="61"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="68" t="s">
         <v>38</v>
       </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="26"/>
+      <c r="E21" s="69"/>
+      <c r="F21" s="69"/>
+      <c r="G21" s="69"/>
+      <c r="H21" s="69"/>
+      <c r="I21" s="70"/>
       <c r="J21" s="2"/>
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
@@ -3015,15 +3019,15 @@
       <c r="Z21" s="3"/>
     </row>
     <row r="22" spans="1:26" ht="24.75" customHeight="1">
-      <c r="A22" s="29"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="33"/>
+      <c r="A22" s="47"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="71"/>
+      <c r="E22" s="71"/>
+      <c r="F22" s="71"/>
+      <c r="G22" s="71"/>
+      <c r="H22" s="71"/>
+      <c r="I22" s="72"/>
       <c r="J22" s="2"/>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
@@ -3043,21 +3047,21 @@
       <c r="Z22" s="3"/>
     </row>
     <row r="23" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A23" s="44" t="s">
+      <c r="A23" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="20"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="39"/>
       <c r="D23" s="38">
         <v>5663000</v>
       </c>
-      <c r="E23" s="20"/>
-      <c r="F23" s="43" t="s">
+      <c r="E23" s="39"/>
+      <c r="F23" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="23"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="42"/>
       <c r="J23" s="2"/>
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
@@ -3077,16 +3081,16 @@
       <c r="Z23" s="3"/>
     </row>
     <row r="24" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A24" s="50" t="s">
+      <c r="A24" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
-      <c r="G24" s="51"/>
-      <c r="H24" s="51"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23"/>
       <c r="I24" s="52"/>
       <c r="J24" s="2">
         <v>4</v>
@@ -3109,23 +3113,23 @@
       <c r="Z24" s="3"/>
     </row>
     <row r="25" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A25" s="45" t="s">
+      <c r="A25" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="46"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="48" t="s">
+      <c r="B25" s="45"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="E25" s="46"/>
-      <c r="F25" s="47"/>
-      <c r="G25" s="17" t="s">
+      <c r="E25" s="45"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="H25" s="39">
+      <c r="H25" s="55">
         <v>3500254256</v>
       </c>
-      <c r="I25" s="40"/>
+      <c r="I25" s="21"/>
       <c r="J25" s="2"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
@@ -3145,19 +3149,19 @@
       <c r="Z25" s="3"/>
     </row>
     <row r="26" spans="1:26" ht="28.5" customHeight="1">
-      <c r="A26" s="29"/>
-      <c r="B26" s="30"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="49"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="17" t="s">
+      <c r="A26" s="47"/>
+      <c r="B26" s="48"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="50"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="H26" s="39">
+      <c r="H26" s="55">
         <v>4500396203</v>
       </c>
-      <c r="I26" s="40"/>
+      <c r="I26" s="21"/>
       <c r="J26" s="2"/>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
@@ -3177,19 +3181,19 @@
       <c r="Z26" s="3"/>
     </row>
     <row r="27" spans="1:26" ht="90" customHeight="1">
-      <c r="A27" s="34" t="s">
+      <c r="A27" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="35"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="41" t="s">
+      <c r="B27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="35"/>
-      <c r="I27" s="40"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="21"/>
       <c r="J27" s="2"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
@@ -3209,21 +3213,21 @@
       <c r="Z27" s="3"/>
     </row>
     <row r="28" spans="1:26" ht="34.5" customHeight="1">
-      <c r="A28" s="37" t="s">
+      <c r="A28" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="20"/>
+      <c r="B28" s="41"/>
+      <c r="C28" s="39"/>
       <c r="D28" s="38">
         <v>33978000</v>
       </c>
-      <c r="E28" s="20"/>
-      <c r="F28" s="42" t="s">
+      <c r="E28" s="39"/>
+      <c r="F28" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="23"/>
+      <c r="G28" s="41"/>
+      <c r="H28" s="41"/>
+      <c r="I28" s="42"/>
       <c r="J28" s="2"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
@@ -3252,7 +3256,7 @@
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
-      <c r="J29" s="8"/>
+      <c r="J29" s="7"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
@@ -3280,7 +3284,7 @@
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
-      <c r="J30" s="8"/>
+      <c r="J30" s="7"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="3"/>
@@ -3308,7 +3312,7 @@
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="8"/>
+      <c r="J31" s="7"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
@@ -3336,7 +3340,7 @@
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="8"/>
+      <c r="J32" s="7"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
@@ -3364,7 +3368,7 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="8"/>
+      <c r="J33" s="7"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
@@ -3392,7 +3396,7 @@
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
-      <c r="J34" s="8"/>
+      <c r="J34" s="7"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
@@ -3420,7 +3424,7 @@
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
-      <c r="J35" s="8"/>
+      <c r="J35" s="7"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
@@ -3448,7 +3452,7 @@
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
-      <c r="J36" s="8"/>
+      <c r="J36" s="7"/>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
@@ -3476,7 +3480,7 @@
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
-      <c r="J37" s="8"/>
+      <c r="J37" s="7"/>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
@@ -3504,7 +3508,7 @@
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
-      <c r="J38" s="8"/>
+      <c r="J38" s="7"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
@@ -3532,7 +3536,7 @@
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
-      <c r="J39" s="8"/>
+      <c r="J39" s="7"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
@@ -3560,7 +3564,7 @@
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
-      <c r="J40" s="8"/>
+      <c r="J40" s="7"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
@@ -3588,7 +3592,7 @@
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
-      <c r="J41" s="8"/>
+      <c r="J41" s="7"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
@@ -3616,7 +3620,7 @@
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
-      <c r="J42" s="8"/>
+      <c r="J42" s="7"/>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
@@ -3644,7 +3648,7 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3"/>
-      <c r="J43" s="8"/>
+      <c r="J43" s="7"/>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
@@ -3672,7 +3676,7 @@
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
       <c r="I44" s="3"/>
-      <c r="J44" s="8"/>
+      <c r="J44" s="7"/>
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3"/>
@@ -3700,7 +3704,7 @@
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
       <c r="I45" s="3"/>
-      <c r="J45" s="8"/>
+      <c r="J45" s="7"/>
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
@@ -3728,7 +3732,7 @@
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
       <c r="I46" s="3"/>
-      <c r="J46" s="8"/>
+      <c r="J46" s="7"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3"/>
@@ -3756,7 +3760,7 @@
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
-      <c r="J47" s="8"/>
+      <c r="J47" s="7"/>
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3"/>
@@ -3784,7 +3788,7 @@
       <c r="G48" s="3"/>
       <c r="H48" s="3"/>
       <c r="I48" s="3"/>
-      <c r="J48" s="8"/>
+      <c r="J48" s="7"/>
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="3"/>
@@ -3812,7 +3816,7 @@
       <c r="G49" s="3"/>
       <c r="H49" s="3"/>
       <c r="I49" s="3"/>
-      <c r="J49" s="8"/>
+      <c r="J49" s="7"/>
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
@@ -3840,7 +3844,7 @@
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
       <c r="I50" s="3"/>
-      <c r="J50" s="8"/>
+      <c r="J50" s="7"/>
       <c r="K50" s="3"/>
       <c r="L50" s="3"/>
       <c r="M50" s="3"/>
@@ -3868,7 +3872,7 @@
       <c r="G51" s="3"/>
       <c r="H51" s="3"/>
       <c r="I51" s="3"/>
-      <c r="J51" s="8"/>
+      <c r="J51" s="7"/>
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3"/>
@@ -3896,7 +3900,7 @@
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
       <c r="I52" s="3"/>
-      <c r="J52" s="8"/>
+      <c r="J52" s="7"/>
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
       <c r="M52" s="3"/>
@@ -3924,7 +3928,7 @@
       <c r="G53" s="3"/>
       <c r="H53" s="3"/>
       <c r="I53" s="3"/>
-      <c r="J53" s="8"/>
+      <c r="J53" s="7"/>
       <c r="K53" s="3"/>
       <c r="L53" s="3"/>
       <c r="M53" s="3"/>
@@ -3952,7 +3956,7 @@
       <c r="G54" s="3"/>
       <c r="H54" s="3"/>
       <c r="I54" s="3"/>
-      <c r="J54" s="8"/>
+      <c r="J54" s="7"/>
       <c r="K54" s="3"/>
       <c r="L54" s="3"/>
       <c r="M54" s="3"/>
@@ -3980,7 +3984,7 @@
       <c r="G55" s="3"/>
       <c r="H55" s="3"/>
       <c r="I55" s="3"/>
-      <c r="J55" s="8"/>
+      <c r="J55" s="7"/>
       <c r="K55" s="3"/>
       <c r="L55" s="3"/>
       <c r="M55" s="3"/>
@@ -4008,7 +4012,7 @@
       <c r="G56" s="3"/>
       <c r="H56" s="3"/>
       <c r="I56" s="3"/>
-      <c r="J56" s="8"/>
+      <c r="J56" s="7"/>
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
       <c r="M56" s="3"/>
@@ -4036,7 +4040,7 @@
       <c r="G57" s="3"/>
       <c r="H57" s="3"/>
       <c r="I57" s="3"/>
-      <c r="J57" s="8"/>
+      <c r="J57" s="7"/>
       <c r="K57" s="3"/>
       <c r="L57" s="3"/>
       <c r="M57" s="3"/>
@@ -4064,7 +4068,7 @@
       <c r="G58" s="3"/>
       <c r="H58" s="3"/>
       <c r="I58" s="3"/>
-      <c r="J58" s="8"/>
+      <c r="J58" s="7"/>
       <c r="K58" s="3"/>
       <c r="L58" s="3"/>
       <c r="M58" s="3"/>
@@ -4092,7 +4096,7 @@
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
       <c r="I59" s="3"/>
-      <c r="J59" s="8"/>
+      <c r="J59" s="7"/>
       <c r="K59" s="3"/>
       <c r="L59" s="3"/>
       <c r="M59" s="3"/>
@@ -4120,7 +4124,7 @@
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
       <c r="I60" s="3"/>
-      <c r="J60" s="8"/>
+      <c r="J60" s="7"/>
       <c r="K60" s="3"/>
       <c r="L60" s="3"/>
       <c r="M60" s="3"/>
@@ -4148,7 +4152,7 @@
       <c r="G61" s="3"/>
       <c r="H61" s="3"/>
       <c r="I61" s="3"/>
-      <c r="J61" s="8"/>
+      <c r="J61" s="7"/>
       <c r="K61" s="3"/>
       <c r="L61" s="3"/>
       <c r="M61" s="3"/>
@@ -4176,7 +4180,7 @@
       <c r="G62" s="3"/>
       <c r="H62" s="3"/>
       <c r="I62" s="3"/>
-      <c r="J62" s="8"/>
+      <c r="J62" s="7"/>
       <c r="K62" s="3"/>
       <c r="L62" s="3"/>
       <c r="M62" s="3"/>
@@ -4204,7 +4208,7 @@
       <c r="G63" s="3"/>
       <c r="H63" s="3"/>
       <c r="I63" s="3"/>
-      <c r="J63" s="8"/>
+      <c r="J63" s="7"/>
       <c r="K63" s="3"/>
       <c r="L63" s="3"/>
       <c r="M63" s="3"/>
@@ -4232,7 +4236,7 @@
       <c r="G64" s="3"/>
       <c r="H64" s="3"/>
       <c r="I64" s="3"/>
-      <c r="J64" s="8"/>
+      <c r="J64" s="7"/>
       <c r="K64" s="3"/>
       <c r="L64" s="3"/>
       <c r="M64" s="3"/>
@@ -4260,7 +4264,7 @@
       <c r="G65" s="3"/>
       <c r="H65" s="3"/>
       <c r="I65" s="3"/>
-      <c r="J65" s="8"/>
+      <c r="J65" s="7"/>
       <c r="K65" s="3"/>
       <c r="L65" s="3"/>
       <c r="M65" s="3"/>
@@ -4288,7 +4292,7 @@
       <c r="G66" s="3"/>
       <c r="H66" s="3"/>
       <c r="I66" s="3"/>
-      <c r="J66" s="8"/>
+      <c r="J66" s="7"/>
       <c r="K66" s="3"/>
       <c r="L66" s="3"/>
       <c r="M66" s="3"/>
@@ -4316,7 +4320,7 @@
       <c r="G67" s="3"/>
       <c r="H67" s="3"/>
       <c r="I67" s="3"/>
-      <c r="J67" s="8"/>
+      <c r="J67" s="7"/>
       <c r="K67" s="3"/>
       <c r="L67" s="3"/>
       <c r="M67" s="3"/>
@@ -4344,7 +4348,7 @@
       <c r="G68" s="3"/>
       <c r="H68" s="3"/>
       <c r="I68" s="3"/>
-      <c r="J68" s="8"/>
+      <c r="J68" s="7"/>
       <c r="K68" s="3"/>
       <c r="L68" s="3"/>
       <c r="M68" s="3"/>
@@ -4372,7 +4376,7 @@
       <c r="G69" s="3"/>
       <c r="H69" s="3"/>
       <c r="I69" s="3"/>
-      <c r="J69" s="8"/>
+      <c r="J69" s="7"/>
       <c r="K69" s="3"/>
       <c r="L69" s="3"/>
       <c r="M69" s="3"/>
@@ -4400,7 +4404,7 @@
       <c r="G70" s="3"/>
       <c r="H70" s="3"/>
       <c r="I70" s="3"/>
-      <c r="J70" s="8"/>
+      <c r="J70" s="7"/>
       <c r="K70" s="3"/>
       <c r="L70" s="3"/>
       <c r="M70" s="3"/>
@@ -4428,7 +4432,7 @@
       <c r="G71" s="3"/>
       <c r="H71" s="3"/>
       <c r="I71" s="3"/>
-      <c r="J71" s="8"/>
+      <c r="J71" s="7"/>
       <c r="K71" s="3"/>
       <c r="L71" s="3"/>
       <c r="M71" s="3"/>
@@ -4456,7 +4460,7 @@
       <c r="G72" s="3"/>
       <c r="H72" s="3"/>
       <c r="I72" s="3"/>
-      <c r="J72" s="8"/>
+      <c r="J72" s="7"/>
       <c r="K72" s="3"/>
       <c r="L72" s="3"/>
       <c r="M72" s="3"/>
@@ -4484,7 +4488,7 @@
       <c r="G73" s="3"/>
       <c r="H73" s="3"/>
       <c r="I73" s="3"/>
-      <c r="J73" s="8"/>
+      <c r="J73" s="7"/>
       <c r="K73" s="3"/>
       <c r="L73" s="3"/>
       <c r="M73" s="3"/>
@@ -4512,7 +4516,7 @@
       <c r="G74" s="3"/>
       <c r="H74" s="3"/>
       <c r="I74" s="3"/>
-      <c r="J74" s="8"/>
+      <c r="J74" s="7"/>
       <c r="K74" s="3"/>
       <c r="L74" s="3"/>
       <c r="M74" s="3"/>
@@ -4540,7 +4544,7 @@
       <c r="G75" s="3"/>
       <c r="H75" s="3"/>
       <c r="I75" s="3"/>
-      <c r="J75" s="8"/>
+      <c r="J75" s="7"/>
       <c r="K75" s="3"/>
       <c r="L75" s="3"/>
       <c r="M75" s="3"/>
@@ -4568,7 +4572,7 @@
       <c r="G76" s="3"/>
       <c r="H76" s="3"/>
       <c r="I76" s="3"/>
-      <c r="J76" s="8"/>
+      <c r="J76" s="7"/>
       <c r="K76" s="3"/>
       <c r="L76" s="3"/>
       <c r="M76" s="3"/>
@@ -4596,7 +4600,7 @@
       <c r="G77" s="3"/>
       <c r="H77" s="3"/>
       <c r="I77" s="3"/>
-      <c r="J77" s="8"/>
+      <c r="J77" s="7"/>
       <c r="K77" s="3"/>
       <c r="L77" s="3"/>
       <c r="M77" s="3"/>
@@ -4624,7 +4628,7 @@
       <c r="G78" s="3"/>
       <c r="H78" s="3"/>
       <c r="I78" s="3"/>
-      <c r="J78" s="8"/>
+      <c r="J78" s="7"/>
       <c r="K78" s="3"/>
       <c r="L78" s="3"/>
       <c r="M78" s="3"/>
@@ -4652,7 +4656,7 @@
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
       <c r="I79" s="3"/>
-      <c r="J79" s="8"/>
+      <c r="J79" s="7"/>
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
       <c r="M79" s="3"/>
@@ -4680,7 +4684,7 @@
       <c r="G80" s="3"/>
       <c r="H80" s="3"/>
       <c r="I80" s="3"/>
-      <c r="J80" s="8"/>
+      <c r="J80" s="7"/>
       <c r="K80" s="3"/>
       <c r="L80" s="3"/>
       <c r="M80" s="3"/>
@@ -4708,7 +4712,7 @@
       <c r="G81" s="3"/>
       <c r="H81" s="3"/>
       <c r="I81" s="3"/>
-      <c r="J81" s="8"/>
+      <c r="J81" s="7"/>
       <c r="K81" s="3"/>
       <c r="L81" s="3"/>
       <c r="M81" s="3"/>
@@ -4736,7 +4740,7 @@
       <c r="G82" s="3"/>
       <c r="H82" s="3"/>
       <c r="I82" s="3"/>
-      <c r="J82" s="8"/>
+      <c r="J82" s="7"/>
       <c r="K82" s="3"/>
       <c r="L82" s="3"/>
       <c r="M82" s="3"/>
@@ -4764,7 +4768,7 @@
       <c r="G83" s="3"/>
       <c r="H83" s="3"/>
       <c r="I83" s="3"/>
-      <c r="J83" s="8"/>
+      <c r="J83" s="7"/>
       <c r="K83" s="3"/>
       <c r="L83" s="3"/>
       <c r="M83" s="3"/>
@@ -4792,7 +4796,7 @@
       <c r="G84" s="3"/>
       <c r="H84" s="3"/>
       <c r="I84" s="3"/>
-      <c r="J84" s="8"/>
+      <c r="J84" s="7"/>
       <c r="K84" s="3"/>
       <c r="L84" s="3"/>
       <c r="M84" s="3"/>
@@ -4820,7 +4824,7 @@
       <c r="G85" s="3"/>
       <c r="H85" s="3"/>
       <c r="I85" s="3"/>
-      <c r="J85" s="8"/>
+      <c r="J85" s="7"/>
       <c r="K85" s="3"/>
       <c r="L85" s="3"/>
       <c r="M85" s="3"/>
@@ -4848,7 +4852,7 @@
       <c r="G86" s="3"/>
       <c r="H86" s="3"/>
       <c r="I86" s="3"/>
-      <c r="J86" s="8"/>
+      <c r="J86" s="7"/>
       <c r="K86" s="3"/>
       <c r="L86" s="3"/>
       <c r="M86" s="3"/>
@@ -4876,7 +4880,7 @@
       <c r="G87" s="3"/>
       <c r="H87" s="3"/>
       <c r="I87" s="3"/>
-      <c r="J87" s="8"/>
+      <c r="J87" s="7"/>
       <c r="K87" s="3"/>
       <c r="L87" s="3"/>
       <c r="M87" s="3"/>
@@ -4904,7 +4908,7 @@
       <c r="G88" s="3"/>
       <c r="H88" s="3"/>
       <c r="I88" s="3"/>
-      <c r="J88" s="8"/>
+      <c r="J88" s="7"/>
       <c r="K88" s="3"/>
       <c r="L88" s="3"/>
       <c r="M88" s="3"/>
@@ -4932,7 +4936,7 @@
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
       <c r="I89" s="3"/>
-      <c r="J89" s="8"/>
+      <c r="J89" s="7"/>
       <c r="K89" s="3"/>
       <c r="L89" s="3"/>
       <c r="M89" s="3"/>
@@ -4960,7 +4964,7 @@
       <c r="G90" s="3"/>
       <c r="H90" s="3"/>
       <c r="I90" s="3"/>
-      <c r="J90" s="8"/>
+      <c r="J90" s="7"/>
       <c r="K90" s="3"/>
       <c r="L90" s="3"/>
       <c r="M90" s="3"/>
@@ -4988,7 +4992,7 @@
       <c r="G91" s="3"/>
       <c r="H91" s="3"/>
       <c r="I91" s="3"/>
-      <c r="J91" s="8"/>
+      <c r="J91" s="7"/>
       <c r="K91" s="3"/>
       <c r="L91" s="3"/>
       <c r="M91" s="3"/>
@@ -5016,7 +5020,7 @@
       <c r="G92" s="3"/>
       <c r="H92" s="3"/>
       <c r="I92" s="3"/>
-      <c r="J92" s="8"/>
+      <c r="J92" s="7"/>
       <c r="K92" s="3"/>
       <c r="L92" s="3"/>
       <c r="M92" s="3"/>
@@ -5044,7 +5048,7 @@
       <c r="G93" s="3"/>
       <c r="H93" s="3"/>
       <c r="I93" s="3"/>
-      <c r="J93" s="8"/>
+      <c r="J93" s="7"/>
       <c r="K93" s="3"/>
       <c r="L93" s="3"/>
       <c r="M93" s="3"/>
@@ -5072,7 +5076,7 @@
       <c r="G94" s="3"/>
       <c r="H94" s="3"/>
       <c r="I94" s="3"/>
-      <c r="J94" s="8"/>
+      <c r="J94" s="7"/>
       <c r="K94" s="3"/>
       <c r="L94" s="3"/>
       <c r="M94" s="3"/>
@@ -5100,7 +5104,7 @@
       <c r="G95" s="3"/>
       <c r="H95" s="3"/>
       <c r="I95" s="3"/>
-      <c r="J95" s="8"/>
+      <c r="J95" s="7"/>
       <c r="K95" s="3"/>
       <c r="L95" s="3"/>
       <c r="M95" s="3"/>
@@ -5128,7 +5132,7 @@
       <c r="G96" s="3"/>
       <c r="H96" s="3"/>
       <c r="I96" s="3"/>
-      <c r="J96" s="8"/>
+      <c r="J96" s="7"/>
       <c r="K96" s="3"/>
       <c r="L96" s="3"/>
       <c r="M96" s="3"/>
@@ -5156,7 +5160,7 @@
       <c r="G97" s="3"/>
       <c r="H97" s="3"/>
       <c r="I97" s="3"/>
-      <c r="J97" s="8"/>
+      <c r="J97" s="7"/>
       <c r="K97" s="3"/>
       <c r="L97" s="3"/>
       <c r="M97" s="3"/>
@@ -5184,7 +5188,7 @@
       <c r="G98" s="3"/>
       <c r="H98" s="3"/>
       <c r="I98" s="3"/>
-      <c r="J98" s="8"/>
+      <c r="J98" s="7"/>
       <c r="K98" s="3"/>
       <c r="L98" s="3"/>
       <c r="M98" s="3"/>
@@ -5212,7 +5216,7 @@
       <c r="G99" s="3"/>
       <c r="H99" s="3"/>
       <c r="I99" s="3"/>
-      <c r="J99" s="8"/>
+      <c r="J99" s="7"/>
       <c r="K99" s="3"/>
       <c r="L99" s="3"/>
       <c r="M99" s="3"/>
@@ -5240,7 +5244,7 @@
       <c r="G100" s="3"/>
       <c r="H100" s="3"/>
       <c r="I100" s="3"/>
-      <c r="J100" s="8"/>
+      <c r="J100" s="7"/>
       <c r="K100" s="3"/>
       <c r="L100" s="3"/>
       <c r="M100" s="3"/>
@@ -5268,7 +5272,7 @@
       <c r="G101" s="3"/>
       <c r="H101" s="3"/>
       <c r="I101" s="3"/>
-      <c r="J101" s="8"/>
+      <c r="J101" s="7"/>
       <c r="K101" s="3"/>
       <c r="L101" s="3"/>
       <c r="M101" s="3"/>
@@ -5296,7 +5300,7 @@
       <c r="G102" s="3"/>
       <c r="H102" s="3"/>
       <c r="I102" s="3"/>
-      <c r="J102" s="8"/>
+      <c r="J102" s="7"/>
       <c r="K102" s="3"/>
       <c r="L102" s="3"/>
       <c r="M102" s="3"/>
@@ -5324,7 +5328,7 @@
       <c r="G103" s="3"/>
       <c r="H103" s="3"/>
       <c r="I103" s="3"/>
-      <c r="J103" s="8"/>
+      <c r="J103" s="7"/>
       <c r="K103" s="3"/>
       <c r="L103" s="3"/>
       <c r="M103" s="3"/>
@@ -5352,7 +5356,7 @@
       <c r="G104" s="3"/>
       <c r="H104" s="3"/>
       <c r="I104" s="3"/>
-      <c r="J104" s="8"/>
+      <c r="J104" s="7"/>
       <c r="K104" s="3"/>
       <c r="L104" s="3"/>
       <c r="M104" s="3"/>
@@ -5380,7 +5384,7 @@
       <c r="G105" s="3"/>
       <c r="H105" s="3"/>
       <c r="I105" s="3"/>
-      <c r="J105" s="8"/>
+      <c r="J105" s="7"/>
       <c r="K105" s="3"/>
       <c r="L105" s="3"/>
       <c r="M105" s="3"/>
@@ -5408,7 +5412,7 @@
       <c r="G106" s="3"/>
       <c r="H106" s="3"/>
       <c r="I106" s="3"/>
-      <c r="J106" s="8"/>
+      <c r="J106" s="7"/>
       <c r="K106" s="3"/>
       <c r="L106" s="3"/>
       <c r="M106" s="3"/>
@@ -5436,7 +5440,7 @@
       <c r="G107" s="3"/>
       <c r="H107" s="3"/>
       <c r="I107" s="3"/>
-      <c r="J107" s="8"/>
+      <c r="J107" s="7"/>
       <c r="K107" s="3"/>
       <c r="L107" s="3"/>
       <c r="M107" s="3"/>
@@ -5464,7 +5468,7 @@
       <c r="G108" s="3"/>
       <c r="H108" s="3"/>
       <c r="I108" s="3"/>
-      <c r="J108" s="8"/>
+      <c r="J108" s="7"/>
       <c r="K108" s="3"/>
       <c r="L108" s="3"/>
       <c r="M108" s="3"/>
@@ -5492,7 +5496,7 @@
       <c r="G109" s="3"/>
       <c r="H109" s="3"/>
       <c r="I109" s="3"/>
-      <c r="J109" s="8"/>
+      <c r="J109" s="7"/>
       <c r="K109" s="3"/>
       <c r="L109" s="3"/>
       <c r="M109" s="3"/>
@@ -5520,7 +5524,7 @@
       <c r="G110" s="3"/>
       <c r="H110" s="3"/>
       <c r="I110" s="3"/>
-      <c r="J110" s="8"/>
+      <c r="J110" s="7"/>
       <c r="K110" s="3"/>
       <c r="L110" s="3"/>
       <c r="M110" s="3"/>
@@ -5548,7 +5552,7 @@
       <c r="G111" s="3"/>
       <c r="H111" s="3"/>
       <c r="I111" s="3"/>
-      <c r="J111" s="8"/>
+      <c r="J111" s="7"/>
       <c r="K111" s="3"/>
       <c r="L111" s="3"/>
       <c r="M111" s="3"/>
@@ -5576,7 +5580,7 @@
       <c r="G112" s="3"/>
       <c r="H112" s="3"/>
       <c r="I112" s="3"/>
-      <c r="J112" s="8"/>
+      <c r="J112" s="7"/>
       <c r="K112" s="3"/>
       <c r="L112" s="3"/>
       <c r="M112" s="3"/>
@@ -5604,7 +5608,7 @@
       <c r="G113" s="3"/>
       <c r="H113" s="3"/>
       <c r="I113" s="3"/>
-      <c r="J113" s="8"/>
+      <c r="J113" s="7"/>
       <c r="K113" s="3"/>
       <c r="L113" s="3"/>
       <c r="M113" s="3"/>
@@ -5632,7 +5636,7 @@
       <c r="G114" s="3"/>
       <c r="H114" s="3"/>
       <c r="I114" s="3"/>
-      <c r="J114" s="8"/>
+      <c r="J114" s="7"/>
       <c r="K114" s="3"/>
       <c r="L114" s="3"/>
       <c r="M114" s="3"/>
@@ -5660,7 +5664,7 @@
       <c r="G115" s="3"/>
       <c r="H115" s="3"/>
       <c r="I115" s="3"/>
-      <c r="J115" s="8"/>
+      <c r="J115" s="7"/>
       <c r="K115" s="3"/>
       <c r="L115" s="3"/>
       <c r="M115" s="3"/>
@@ -5688,7 +5692,7 @@
       <c r="G116" s="3"/>
       <c r="H116" s="3"/>
       <c r="I116" s="3"/>
-      <c r="J116" s="8"/>
+      <c r="J116" s="7"/>
       <c r="K116" s="3"/>
       <c r="L116" s="3"/>
       <c r="M116" s="3"/>
@@ -5716,7 +5720,7 @@
       <c r="G117" s="3"/>
       <c r="H117" s="3"/>
       <c r="I117" s="3"/>
-      <c r="J117" s="8"/>
+      <c r="J117" s="7"/>
       <c r="K117" s="3"/>
       <c r="L117" s="3"/>
       <c r="M117" s="3"/>
@@ -5744,7 +5748,7 @@
       <c r="G118" s="3"/>
       <c r="H118" s="3"/>
       <c r="I118" s="3"/>
-      <c r="J118" s="8"/>
+      <c r="J118" s="7"/>
       <c r="K118" s="3"/>
       <c r="L118" s="3"/>
       <c r="M118" s="3"/>
@@ -5772,7 +5776,7 @@
       <c r="G119" s="3"/>
       <c r="H119" s="3"/>
       <c r="I119" s="3"/>
-      <c r="J119" s="8"/>
+      <c r="J119" s="7"/>
       <c r="K119" s="3"/>
       <c r="L119" s="3"/>
       <c r="M119" s="3"/>
@@ -5800,7 +5804,7 @@
       <c r="G120" s="3"/>
       <c r="H120" s="3"/>
       <c r="I120" s="3"/>
-      <c r="J120" s="8"/>
+      <c r="J120" s="7"/>
       <c r="K120" s="3"/>
       <c r="L120" s="3"/>
       <c r="M120" s="3"/>
@@ -5828,7 +5832,7 @@
       <c r="G121" s="3"/>
       <c r="H121" s="3"/>
       <c r="I121" s="3"/>
-      <c r="J121" s="8"/>
+      <c r="J121" s="7"/>
       <c r="K121" s="3"/>
       <c r="L121" s="3"/>
       <c r="M121" s="3"/>
@@ -5856,7 +5860,7 @@
       <c r="G122" s="3"/>
       <c r="H122" s="3"/>
       <c r="I122" s="3"/>
-      <c r="J122" s="8"/>
+      <c r="J122" s="7"/>
       <c r="K122" s="3"/>
       <c r="L122" s="3"/>
       <c r="M122" s="3"/>
@@ -5884,7 +5888,7 @@
       <c r="G123" s="3"/>
       <c r="H123" s="3"/>
       <c r="I123" s="3"/>
-      <c r="J123" s="8"/>
+      <c r="J123" s="7"/>
       <c r="K123" s="3"/>
       <c r="L123" s="3"/>
       <c r="M123" s="3"/>
@@ -5912,7 +5916,7 @@
       <c r="G124" s="3"/>
       <c r="H124" s="3"/>
       <c r="I124" s="3"/>
-      <c r="J124" s="8"/>
+      <c r="J124" s="7"/>
       <c r="K124" s="3"/>
       <c r="L124" s="3"/>
       <c r="M124" s="3"/>
@@ -5940,7 +5944,7 @@
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
       <c r="I125" s="3"/>
-      <c r="J125" s="8"/>
+      <c r="J125" s="7"/>
       <c r="K125" s="3"/>
       <c r="L125" s="3"/>
       <c r="M125" s="3"/>
@@ -5968,7 +5972,7 @@
       <c r="G126" s="3"/>
       <c r="H126" s="3"/>
       <c r="I126" s="3"/>
-      <c r="J126" s="8"/>
+      <c r="J126" s="7"/>
       <c r="K126" s="3"/>
       <c r="L126" s="3"/>
       <c r="M126" s="3"/>
@@ -5996,7 +6000,7 @@
       <c r="G127" s="3"/>
       <c r="H127" s="3"/>
       <c r="I127" s="3"/>
-      <c r="J127" s="8"/>
+      <c r="J127" s="7"/>
       <c r="K127" s="3"/>
       <c r="L127" s="3"/>
       <c r="M127" s="3"/>
@@ -6024,7 +6028,7 @@
       <c r="G128" s="3"/>
       <c r="H128" s="3"/>
       <c r="I128" s="3"/>
-      <c r="J128" s="8"/>
+      <c r="J128" s="7"/>
       <c r="K128" s="3"/>
       <c r="L128" s="3"/>
       <c r="M128" s="3"/>
@@ -6052,7 +6056,7 @@
       <c r="G129" s="3"/>
       <c r="H129" s="3"/>
       <c r="I129" s="3"/>
-      <c r="J129" s="8"/>
+      <c r="J129" s="7"/>
       <c r="K129" s="3"/>
       <c r="L129" s="3"/>
       <c r="M129" s="3"/>
@@ -6080,7 +6084,7 @@
       <c r="G130" s="3"/>
       <c r="H130" s="3"/>
       <c r="I130" s="3"/>
-      <c r="J130" s="8"/>
+      <c r="J130" s="7"/>
       <c r="K130" s="3"/>
       <c r="L130" s="3"/>
       <c r="M130" s="3"/>
@@ -6108,7 +6112,7 @@
       <c r="G131" s="3"/>
       <c r="H131" s="3"/>
       <c r="I131" s="3"/>
-      <c r="J131" s="8"/>
+      <c r="J131" s="7"/>
       <c r="K131" s="3"/>
       <c r="L131" s="3"/>
       <c r="M131" s="3"/>
@@ -6136,7 +6140,7 @@
       <c r="G132" s="3"/>
       <c r="H132" s="3"/>
       <c r="I132" s="3"/>
-      <c r="J132" s="8"/>
+      <c r="J132" s="7"/>
       <c r="K132" s="3"/>
       <c r="L132" s="3"/>
       <c r="M132" s="3"/>
@@ -6164,7 +6168,7 @@
       <c r="G133" s="3"/>
       <c r="H133" s="3"/>
       <c r="I133" s="3"/>
-      <c r="J133" s="8"/>
+      <c r="J133" s="7"/>
       <c r="K133" s="3"/>
       <c r="L133" s="3"/>
       <c r="M133" s="3"/>
@@ -6192,7 +6196,7 @@
       <c r="G134" s="3"/>
       <c r="H134" s="3"/>
       <c r="I134" s="3"/>
-      <c r="J134" s="8"/>
+      <c r="J134" s="7"/>
       <c r="K134" s="3"/>
       <c r="L134" s="3"/>
       <c r="M134" s="3"/>
@@ -6220,7 +6224,7 @@
       <c r="G135" s="3"/>
       <c r="H135" s="3"/>
       <c r="I135" s="3"/>
-      <c r="J135" s="8"/>
+      <c r="J135" s="7"/>
       <c r="K135" s="3"/>
       <c r="L135" s="3"/>
       <c r="M135" s="3"/>
@@ -6248,7 +6252,7 @@
       <c r="G136" s="3"/>
       <c r="H136" s="3"/>
       <c r="I136" s="3"/>
-      <c r="J136" s="8"/>
+      <c r="J136" s="7"/>
       <c r="K136" s="3"/>
       <c r="L136" s="3"/>
       <c r="M136" s="3"/>
@@ -6276,7 +6280,7 @@
       <c r="G137" s="3"/>
       <c r="H137" s="3"/>
       <c r="I137" s="3"/>
-      <c r="J137" s="8"/>
+      <c r="J137" s="7"/>
       <c r="K137" s="3"/>
       <c r="L137" s="3"/>
       <c r="M137" s="3"/>
@@ -6304,7 +6308,7 @@
       <c r="G138" s="3"/>
       <c r="H138" s="3"/>
       <c r="I138" s="3"/>
-      <c r="J138" s="8"/>
+      <c r="J138" s="7"/>
       <c r="K138" s="3"/>
       <c r="L138" s="3"/>
       <c r="M138" s="3"/>
@@ -6332,7 +6336,7 @@
       <c r="G139" s="3"/>
       <c r="H139" s="3"/>
       <c r="I139" s="3"/>
-      <c r="J139" s="8"/>
+      <c r="J139" s="7"/>
       <c r="K139" s="3"/>
       <c r="L139" s="3"/>
       <c r="M139" s="3"/>
@@ -6360,7 +6364,7 @@
       <c r="G140" s="3"/>
       <c r="H140" s="3"/>
       <c r="I140" s="3"/>
-      <c r="J140" s="8"/>
+      <c r="J140" s="7"/>
       <c r="K140" s="3"/>
       <c r="L140" s="3"/>
       <c r="M140" s="3"/>
@@ -6388,7 +6392,7 @@
       <c r="G141" s="3"/>
       <c r="H141" s="3"/>
       <c r="I141" s="3"/>
-      <c r="J141" s="8"/>
+      <c r="J141" s="7"/>
       <c r="K141" s="3"/>
       <c r="L141" s="3"/>
       <c r="M141" s="3"/>
@@ -6416,7 +6420,7 @@
       <c r="G142" s="3"/>
       <c r="H142" s="3"/>
       <c r="I142" s="3"/>
-      <c r="J142" s="8"/>
+      <c r="J142" s="7"/>
       <c r="K142" s="3"/>
       <c r="L142" s="3"/>
       <c r="M142" s="3"/>
@@ -6444,7 +6448,7 @@
       <c r="G143" s="3"/>
       <c r="H143" s="3"/>
       <c r="I143" s="3"/>
-      <c r="J143" s="8"/>
+      <c r="J143" s="7"/>
       <c r="K143" s="3"/>
       <c r="L143" s="3"/>
       <c r="M143" s="3"/>
@@ -6472,7 +6476,7 @@
       <c r="G144" s="3"/>
       <c r="H144" s="3"/>
       <c r="I144" s="3"/>
-      <c r="J144" s="8"/>
+      <c r="J144" s="7"/>
       <c r="K144" s="3"/>
       <c r="L144" s="3"/>
       <c r="M144" s="3"/>
@@ -6500,7 +6504,7 @@
       <c r="G145" s="3"/>
       <c r="H145" s="3"/>
       <c r="I145" s="3"/>
-      <c r="J145" s="8"/>
+      <c r="J145" s="7"/>
       <c r="K145" s="3"/>
       <c r="L145" s="3"/>
       <c r="M145" s="3"/>
@@ -6528,7 +6532,7 @@
       <c r="G146" s="3"/>
       <c r="H146" s="3"/>
       <c r="I146" s="3"/>
-      <c r="J146" s="8"/>
+      <c r="J146" s="7"/>
       <c r="K146" s="3"/>
       <c r="L146" s="3"/>
       <c r="M146" s="3"/>
@@ -6556,7 +6560,7 @@
       <c r="G147" s="3"/>
       <c r="H147" s="3"/>
       <c r="I147" s="3"/>
-      <c r="J147" s="8"/>
+      <c r="J147" s="7"/>
       <c r="K147" s="3"/>
       <c r="L147" s="3"/>
       <c r="M147" s="3"/>
@@ -6584,7 +6588,7 @@
       <c r="G148" s="3"/>
       <c r="H148" s="3"/>
       <c r="I148" s="3"/>
-      <c r="J148" s="8"/>
+      <c r="J148" s="7"/>
       <c r="K148" s="3"/>
       <c r="L148" s="3"/>
       <c r="M148" s="3"/>
@@ -6612,7 +6616,7 @@
       <c r="G149" s="3"/>
       <c r="H149" s="3"/>
       <c r="I149" s="3"/>
-      <c r="J149" s="8"/>
+      <c r="J149" s="7"/>
       <c r="K149" s="3"/>
       <c r="L149" s="3"/>
       <c r="M149" s="3"/>
@@ -6640,7 +6644,7 @@
       <c r="G150" s="3"/>
       <c r="H150" s="3"/>
       <c r="I150" s="3"/>
-      <c r="J150" s="8"/>
+      <c r="J150" s="7"/>
       <c r="K150" s="3"/>
       <c r="L150" s="3"/>
       <c r="M150" s="3"/>
@@ -6668,7 +6672,7 @@
       <c r="G151" s="3"/>
       <c r="H151" s="3"/>
       <c r="I151" s="3"/>
-      <c r="J151" s="8"/>
+      <c r="J151" s="7"/>
       <c r="K151" s="3"/>
       <c r="L151" s="3"/>
       <c r="M151" s="3"/>
@@ -6696,7 +6700,7 @@
       <c r="G152" s="3"/>
       <c r="H152" s="3"/>
       <c r="I152" s="3"/>
-      <c r="J152" s="8"/>
+      <c r="J152" s="7"/>
       <c r="K152" s="3"/>
       <c r="L152" s="3"/>
       <c r="M152" s="3"/>
@@ -6724,7 +6728,7 @@
       <c r="G153" s="3"/>
       <c r="H153" s="3"/>
       <c r="I153" s="3"/>
-      <c r="J153" s="8"/>
+      <c r="J153" s="7"/>
       <c r="K153" s="3"/>
       <c r="L153" s="3"/>
       <c r="M153" s="3"/>
@@ -6752,7 +6756,7 @@
       <c r="G154" s="3"/>
       <c r="H154" s="3"/>
       <c r="I154" s="3"/>
-      <c r="J154" s="8"/>
+      <c r="J154" s="7"/>
       <c r="K154" s="3"/>
       <c r="L154" s="3"/>
       <c r="M154" s="3"/>
@@ -6780,7 +6784,7 @@
       <c r="G155" s="3"/>
       <c r="H155" s="3"/>
       <c r="I155" s="3"/>
-      <c r="J155" s="8"/>
+      <c r="J155" s="7"/>
       <c r="K155" s="3"/>
       <c r="L155" s="3"/>
       <c r="M155" s="3"/>
@@ -6808,7 +6812,7 @@
       <c r="G156" s="3"/>
       <c r="H156" s="3"/>
       <c r="I156" s="3"/>
-      <c r="J156" s="8"/>
+      <c r="J156" s="7"/>
       <c r="K156" s="3"/>
       <c r="L156" s="3"/>
       <c r="M156" s="3"/>
@@ -6836,7 +6840,7 @@
       <c r="G157" s="3"/>
       <c r="H157" s="3"/>
       <c r="I157" s="3"/>
-      <c r="J157" s="8"/>
+      <c r="J157" s="7"/>
       <c r="K157" s="3"/>
       <c r="L157" s="3"/>
       <c r="M157" s="3"/>
@@ -6864,7 +6868,7 @@
       <c r="G158" s="3"/>
       <c r="H158" s="3"/>
       <c r="I158" s="3"/>
-      <c r="J158" s="8"/>
+      <c r="J158" s="7"/>
       <c r="K158" s="3"/>
       <c r="L158" s="3"/>
       <c r="M158" s="3"/>
@@ -6892,7 +6896,7 @@
       <c r="G159" s="3"/>
       <c r="H159" s="3"/>
       <c r="I159" s="3"/>
-      <c r="J159" s="8"/>
+      <c r="J159" s="7"/>
       <c r="K159" s="3"/>
       <c r="L159" s="3"/>
       <c r="M159" s="3"/>
@@ -6920,7 +6924,7 @@
       <c r="G160" s="3"/>
       <c r="H160" s="3"/>
       <c r="I160" s="3"/>
-      <c r="J160" s="8"/>
+      <c r="J160" s="7"/>
       <c r="K160" s="3"/>
       <c r="L160" s="3"/>
       <c r="M160" s="3"/>
@@ -6948,7 +6952,7 @@
       <c r="G161" s="3"/>
       <c r="H161" s="3"/>
       <c r="I161" s="3"/>
-      <c r="J161" s="8"/>
+      <c r="J161" s="7"/>
       <c r="K161" s="3"/>
       <c r="L161" s="3"/>
       <c r="M161" s="3"/>
@@ -6976,7 +6980,7 @@
       <c r="G162" s="3"/>
       <c r="H162" s="3"/>
       <c r="I162" s="3"/>
-      <c r="J162" s="8"/>
+      <c r="J162" s="7"/>
       <c r="K162" s="3"/>
       <c r="L162" s="3"/>
       <c r="M162" s="3"/>
@@ -7004,7 +7008,7 @@
       <c r="G163" s="3"/>
       <c r="H163" s="3"/>
       <c r="I163" s="3"/>
-      <c r="J163" s="8"/>
+      <c r="J163" s="7"/>
       <c r="K163" s="3"/>
       <c r="L163" s="3"/>
       <c r="M163" s="3"/>
@@ -7032,7 +7036,7 @@
       <c r="G164" s="3"/>
       <c r="H164" s="3"/>
       <c r="I164" s="3"/>
-      <c r="J164" s="8"/>
+      <c r="J164" s="7"/>
       <c r="K164" s="3"/>
       <c r="L164" s="3"/>
       <c r="M164" s="3"/>
@@ -7060,7 +7064,7 @@
       <c r="G165" s="3"/>
       <c r="H165" s="3"/>
       <c r="I165" s="3"/>
-      <c r="J165" s="8"/>
+      <c r="J165" s="7"/>
       <c r="K165" s="3"/>
       <c r="L165" s="3"/>
       <c r="M165" s="3"/>
@@ -7088,7 +7092,7 @@
       <c r="G166" s="3"/>
       <c r="H166" s="3"/>
       <c r="I166" s="3"/>
-      <c r="J166" s="8"/>
+      <c r="J166" s="7"/>
       <c r="K166" s="3"/>
       <c r="L166" s="3"/>
       <c r="M166" s="3"/>
@@ -7116,7 +7120,7 @@
       <c r="G167" s="3"/>
       <c r="H167" s="3"/>
       <c r="I167" s="3"/>
-      <c r="J167" s="8"/>
+      <c r="J167" s="7"/>
       <c r="K167" s="3"/>
       <c r="L167" s="3"/>
       <c r="M167" s="3"/>
@@ -7144,7 +7148,7 @@
       <c r="G168" s="3"/>
       <c r="H168" s="3"/>
       <c r="I168" s="3"/>
-      <c r="J168" s="8"/>
+      <c r="J168" s="7"/>
       <c r="K168" s="3"/>
       <c r="L168" s="3"/>
       <c r="M168" s="3"/>
@@ -7172,7 +7176,7 @@
       <c r="G169" s="3"/>
       <c r="H169" s="3"/>
       <c r="I169" s="3"/>
-      <c r="J169" s="8"/>
+      <c r="J169" s="7"/>
       <c r="K169" s="3"/>
       <c r="L169" s="3"/>
       <c r="M169" s="3"/>
@@ -7200,7 +7204,7 @@
       <c r="G170" s="3"/>
       <c r="H170" s="3"/>
       <c r="I170" s="3"/>
-      <c r="J170" s="8"/>
+      <c r="J170" s="7"/>
       <c r="K170" s="3"/>
       <c r="L170" s="3"/>
       <c r="M170" s="3"/>
@@ -7228,7 +7232,7 @@
       <c r="G171" s="3"/>
       <c r="H171" s="3"/>
       <c r="I171" s="3"/>
-      <c r="J171" s="8"/>
+      <c r="J171" s="7"/>
       <c r="K171" s="3"/>
       <c r="L171" s="3"/>
       <c r="M171" s="3"/>
@@ -7256,7 +7260,7 @@
       <c r="G172" s="3"/>
       <c r="H172" s="3"/>
       <c r="I172" s="3"/>
-      <c r="J172" s="8"/>
+      <c r="J172" s="7"/>
       <c r="K172" s="3"/>
       <c r="L172" s="3"/>
       <c r="M172" s="3"/>
@@ -7284,7 +7288,7 @@
       <c r="G173" s="3"/>
       <c r="H173" s="3"/>
       <c r="I173" s="3"/>
-      <c r="J173" s="8"/>
+      <c r="J173" s="7"/>
       <c r="K173" s="3"/>
       <c r="L173" s="3"/>
       <c r="M173" s="3"/>
@@ -7312,7 +7316,7 @@
       <c r="G174" s="3"/>
       <c r="H174" s="3"/>
       <c r="I174" s="3"/>
-      <c r="J174" s="8"/>
+      <c r="J174" s="7"/>
       <c r="K174" s="3"/>
       <c r="L174" s="3"/>
       <c r="M174" s="3"/>
@@ -7340,7 +7344,7 @@
       <c r="G175" s="3"/>
       <c r="H175" s="3"/>
       <c r="I175" s="3"/>
-      <c r="J175" s="8"/>
+      <c r="J175" s="7"/>
       <c r="K175" s="3"/>
       <c r="L175" s="3"/>
       <c r="M175" s="3"/>
@@ -7368,7 +7372,7 @@
       <c r="G176" s="3"/>
       <c r="H176" s="3"/>
       <c r="I176" s="3"/>
-      <c r="J176" s="8"/>
+      <c r="J176" s="7"/>
       <c r="K176" s="3"/>
       <c r="L176" s="3"/>
       <c r="M176" s="3"/>
@@ -7396,7 +7400,7 @@
       <c r="G177" s="3"/>
       <c r="H177" s="3"/>
       <c r="I177" s="3"/>
-      <c r="J177" s="8"/>
+      <c r="J177" s="7"/>
       <c r="K177" s="3"/>
       <c r="L177" s="3"/>
       <c r="M177" s="3"/>
@@ -7424,7 +7428,7 @@
       <c r="G178" s="3"/>
       <c r="H178" s="3"/>
       <c r="I178" s="3"/>
-      <c r="J178" s="8"/>
+      <c r="J178" s="7"/>
       <c r="K178" s="3"/>
       <c r="L178" s="3"/>
       <c r="M178" s="3"/>
@@ -7452,7 +7456,7 @@
       <c r="G179" s="3"/>
       <c r="H179" s="3"/>
       <c r="I179" s="3"/>
-      <c r="J179" s="8"/>
+      <c r="J179" s="7"/>
       <c r="K179" s="3"/>
       <c r="L179" s="3"/>
       <c r="M179" s="3"/>
@@ -7480,7 +7484,7 @@
       <c r="G180" s="3"/>
       <c r="H180" s="3"/>
       <c r="I180" s="3"/>
-      <c r="J180" s="8"/>
+      <c r="J180" s="7"/>
       <c r="K180" s="3"/>
       <c r="L180" s="3"/>
       <c r="M180" s="3"/>
@@ -7508,7 +7512,7 @@
       <c r="G181" s="3"/>
       <c r="H181" s="3"/>
       <c r="I181" s="3"/>
-      <c r="J181" s="8"/>
+      <c r="J181" s="7"/>
       <c r="K181" s="3"/>
       <c r="L181" s="3"/>
       <c r="M181" s="3"/>
@@ -7536,7 +7540,7 @@
       <c r="G182" s="3"/>
       <c r="H182" s="3"/>
       <c r="I182" s="3"/>
-      <c r="J182" s="8"/>
+      <c r="J182" s="7"/>
       <c r="K182" s="3"/>
       <c r="L182" s="3"/>
       <c r="M182" s="3"/>
@@ -7564,7 +7568,7 @@
       <c r="G183" s="3"/>
       <c r="H183" s="3"/>
       <c r="I183" s="3"/>
-      <c r="J183" s="8"/>
+      <c r="J183" s="7"/>
       <c r="K183" s="3"/>
       <c r="L183" s="3"/>
       <c r="M183" s="3"/>
@@ -7592,7 +7596,7 @@
       <c r="G184" s="3"/>
       <c r="H184" s="3"/>
       <c r="I184" s="3"/>
-      <c r="J184" s="8"/>
+      <c r="J184" s="7"/>
       <c r="K184" s="3"/>
       <c r="L184" s="3"/>
       <c r="M184" s="3"/>
@@ -7620,7 +7624,7 @@
       <c r="G185" s="3"/>
       <c r="H185" s="3"/>
       <c r="I185" s="3"/>
-      <c r="J185" s="8"/>
+      <c r="J185" s="7"/>
       <c r="K185" s="3"/>
       <c r="L185" s="3"/>
       <c r="M185" s="3"/>
@@ -7648,7 +7652,7 @@
       <c r="G186" s="3"/>
       <c r="H186" s="3"/>
       <c r="I186" s="3"/>
-      <c r="J186" s="8"/>
+      <c r="J186" s="7"/>
       <c r="K186" s="3"/>
       <c r="L186" s="3"/>
       <c r="M186" s="3"/>
@@ -7676,7 +7680,7 @@
       <c r="G187" s="3"/>
       <c r="H187" s="3"/>
       <c r="I187" s="3"/>
-      <c r="J187" s="8"/>
+      <c r="J187" s="7"/>
       <c r="K187" s="3"/>
       <c r="L187" s="3"/>
       <c r="M187" s="3"/>
@@ -7704,7 +7708,7 @@
       <c r="G188" s="3"/>
       <c r="H188" s="3"/>
       <c r="I188" s="3"/>
-      <c r="J188" s="8"/>
+      <c r="J188" s="7"/>
       <c r="K188" s="3"/>
       <c r="L188" s="3"/>
       <c r="M188" s="3"/>
@@ -7732,7 +7736,7 @@
       <c r="G189" s="3"/>
       <c r="H189" s="3"/>
       <c r="I189" s="3"/>
-      <c r="J189" s="8"/>
+      <c r="J189" s="7"/>
       <c r="K189" s="3"/>
       <c r="L189" s="3"/>
       <c r="M189" s="3"/>
@@ -7760,7 +7764,7 @@
       <c r="G190" s="3"/>
       <c r="H190" s="3"/>
       <c r="I190" s="3"/>
-      <c r="J190" s="8"/>
+      <c r="J190" s="7"/>
       <c r="K190" s="3"/>
       <c r="L190" s="3"/>
       <c r="M190" s="3"/>
@@ -7788,7 +7792,7 @@
       <c r="G191" s="3"/>
       <c r="H191" s="3"/>
       <c r="I191" s="3"/>
-      <c r="J191" s="8"/>
+      <c r="J191" s="7"/>
       <c r="K191" s="3"/>
       <c r="L191" s="3"/>
       <c r="M191" s="3"/>
@@ -7816,7 +7820,7 @@
       <c r="G192" s="3"/>
       <c r="H192" s="3"/>
       <c r="I192" s="3"/>
-      <c r="J192" s="8"/>
+      <c r="J192" s="7"/>
       <c r="K192" s="3"/>
       <c r="L192" s="3"/>
       <c r="M192" s="3"/>
@@ -7844,7 +7848,7 @@
       <c r="G193" s="3"/>
       <c r="H193" s="3"/>
       <c r="I193" s="3"/>
-      <c r="J193" s="8"/>
+      <c r="J193" s="7"/>
       <c r="K193" s="3"/>
       <c r="L193" s="3"/>
       <c r="M193" s="3"/>
@@ -7872,7 +7876,7 @@
       <c r="G194" s="3"/>
       <c r="H194" s="3"/>
       <c r="I194" s="3"/>
-      <c r="J194" s="8"/>
+      <c r="J194" s="7"/>
       <c r="K194" s="3"/>
       <c r="L194" s="3"/>
       <c r="M194" s="3"/>
@@ -7900,7 +7904,7 @@
       <c r="G195" s="3"/>
       <c r="H195" s="3"/>
       <c r="I195" s="3"/>
-      <c r="J195" s="8"/>
+      <c r="J195" s="7"/>
       <c r="K195" s="3"/>
       <c r="L195" s="3"/>
       <c r="M195" s="3"/>
@@ -7928,7 +7932,7 @@
       <c r="G196" s="3"/>
       <c r="H196" s="3"/>
       <c r="I196" s="3"/>
-      <c r="J196" s="8"/>
+      <c r="J196" s="7"/>
       <c r="K196" s="3"/>
       <c r="L196" s="3"/>
       <c r="M196" s="3"/>
@@ -7956,7 +7960,7 @@
       <c r="G197" s="3"/>
       <c r="H197" s="3"/>
       <c r="I197" s="3"/>
-      <c r="J197" s="8"/>
+      <c r="J197" s="7"/>
       <c r="K197" s="3"/>
       <c r="L197" s="3"/>
       <c r="M197" s="3"/>
@@ -7984,7 +7988,7 @@
       <c r="G198" s="3"/>
       <c r="H198" s="3"/>
       <c r="I198" s="3"/>
-      <c r="J198" s="8"/>
+      <c r="J198" s="7"/>
       <c r="K198" s="3"/>
       <c r="L198" s="3"/>
       <c r="M198" s="3"/>
@@ -8012,7 +8016,7 @@
       <c r="G199" s="3"/>
       <c r="H199" s="3"/>
       <c r="I199" s="3"/>
-      <c r="J199" s="8"/>
+      <c r="J199" s="7"/>
       <c r="K199" s="3"/>
       <c r="L199" s="3"/>
       <c r="M199" s="3"/>
@@ -8040,7 +8044,7 @@
       <c r="G200" s="3"/>
       <c r="H200" s="3"/>
       <c r="I200" s="3"/>
-      <c r="J200" s="8"/>
+      <c r="J200" s="7"/>
       <c r="K200" s="3"/>
       <c r="L200" s="3"/>
       <c r="M200" s="3"/>
@@ -8068,7 +8072,7 @@
       <c r="G201" s="3"/>
       <c r="H201" s="3"/>
       <c r="I201" s="3"/>
-      <c r="J201" s="8"/>
+      <c r="J201" s="7"/>
       <c r="K201" s="3"/>
       <c r="L201" s="3"/>
       <c r="M201" s="3"/>
@@ -8096,7 +8100,7 @@
       <c r="G202" s="3"/>
       <c r="H202" s="3"/>
       <c r="I202" s="3"/>
-      <c r="J202" s="8"/>
+      <c r="J202" s="7"/>
       <c r="K202" s="3"/>
       <c r="L202" s="3"/>
       <c r="M202" s="3"/>
@@ -8124,7 +8128,7 @@
       <c r="G203" s="3"/>
       <c r="H203" s="3"/>
       <c r="I203" s="3"/>
-      <c r="J203" s="8"/>
+      <c r="J203" s="7"/>
       <c r="K203" s="3"/>
       <c r="L203" s="3"/>
       <c r="M203" s="3"/>
@@ -8152,7 +8156,7 @@
       <c r="G204" s="3"/>
       <c r="H204" s="3"/>
       <c r="I204" s="3"/>
-      <c r="J204" s="8"/>
+      <c r="J204" s="7"/>
       <c r="K204" s="3"/>
       <c r="L204" s="3"/>
       <c r="M204" s="3"/>
@@ -8180,7 +8184,7 @@
       <c r="G205" s="3"/>
       <c r="H205" s="3"/>
       <c r="I205" s="3"/>
-      <c r="J205" s="8"/>
+      <c r="J205" s="7"/>
       <c r="K205" s="3"/>
       <c r="L205" s="3"/>
       <c r="M205" s="3"/>
@@ -8208,7 +8212,7 @@
       <c r="G206" s="3"/>
       <c r="H206" s="3"/>
       <c r="I206" s="3"/>
-      <c r="J206" s="8"/>
+      <c r="J206" s="7"/>
       <c r="K206" s="3"/>
       <c r="L206" s="3"/>
       <c r="M206" s="3"/>
@@ -8236,7 +8240,7 @@
       <c r="G207" s="3"/>
       <c r="H207" s="3"/>
       <c r="I207" s="3"/>
-      <c r="J207" s="8"/>
+      <c r="J207" s="7"/>
       <c r="K207" s="3"/>
       <c r="L207" s="3"/>
       <c r="M207" s="3"/>
@@ -8264,7 +8268,7 @@
       <c r="G208" s="3"/>
       <c r="H208" s="3"/>
       <c r="I208" s="3"/>
-      <c r="J208" s="8"/>
+      <c r="J208" s="7"/>
       <c r="K208" s="3"/>
       <c r="L208" s="3"/>
       <c r="M208" s="3"/>
@@ -8292,7 +8296,7 @@
       <c r="G209" s="3"/>
       <c r="H209" s="3"/>
       <c r="I209" s="3"/>
-      <c r="J209" s="8"/>
+      <c r="J209" s="7"/>
       <c r="K209" s="3"/>
       <c r="L209" s="3"/>
       <c r="M209" s="3"/>
@@ -8320,7 +8324,7 @@
       <c r="G210" s="3"/>
       <c r="H210" s="3"/>
       <c r="I210" s="3"/>
-      <c r="J210" s="8"/>
+      <c r="J210" s="7"/>
       <c r="K210" s="3"/>
       <c r="L210" s="3"/>
       <c r="M210" s="3"/>
@@ -8348,7 +8352,7 @@
       <c r="G211" s="3"/>
       <c r="H211" s="3"/>
       <c r="I211" s="3"/>
-      <c r="J211" s="8"/>
+      <c r="J211" s="7"/>
       <c r="K211" s="3"/>
       <c r="L211" s="3"/>
       <c r="M211" s="3"/>
@@ -8376,7 +8380,7 @@
       <c r="G212" s="3"/>
       <c r="H212" s="3"/>
       <c r="I212" s="3"/>
-      <c r="J212" s="8"/>
+      <c r="J212" s="7"/>
       <c r="K212" s="3"/>
       <c r="L212" s="3"/>
       <c r="M212" s="3"/>
@@ -8404,7 +8408,7 @@
       <c r="G213" s="3"/>
       <c r="H213" s="3"/>
       <c r="I213" s="3"/>
-      <c r="J213" s="8"/>
+      <c r="J213" s="7"/>
       <c r="K213" s="3"/>
       <c r="L213" s="3"/>
       <c r="M213" s="3"/>
@@ -8432,7 +8436,7 @@
       <c r="G214" s="3"/>
       <c r="H214" s="3"/>
       <c r="I214" s="3"/>
-      <c r="J214" s="8"/>
+      <c r="J214" s="7"/>
       <c r="K214" s="3"/>
       <c r="L214" s="3"/>
       <c r="M214" s="3"/>
@@ -8460,7 +8464,7 @@
       <c r="G215" s="3"/>
       <c r="H215" s="3"/>
       <c r="I215" s="3"/>
-      <c r="J215" s="8"/>
+      <c r="J215" s="7"/>
       <c r="K215" s="3"/>
       <c r="L215" s="3"/>
       <c r="M215" s="3"/>
@@ -8488,7 +8492,7 @@
       <c r="G216" s="3"/>
       <c r="H216" s="3"/>
       <c r="I216" s="3"/>
-      <c r="J216" s="8"/>
+      <c r="J216" s="7"/>
       <c r="K216" s="3"/>
       <c r="L216" s="3"/>
       <c r="M216" s="3"/>
@@ -8516,7 +8520,7 @@
       <c r="G217" s="3"/>
       <c r="H217" s="3"/>
       <c r="I217" s="3"/>
-      <c r="J217" s="8"/>
+      <c r="J217" s="7"/>
       <c r="K217" s="3"/>
       <c r="L217" s="3"/>
       <c r="M217" s="3"/>
@@ -8544,7 +8548,7 @@
       <c r="G218" s="3"/>
       <c r="H218" s="3"/>
       <c r="I218" s="3"/>
-      <c r="J218" s="8"/>
+      <c r="J218" s="7"/>
       <c r="K218" s="3"/>
       <c r="L218" s="3"/>
       <c r="M218" s="3"/>
@@ -8572,7 +8576,7 @@
       <c r="G219" s="3"/>
       <c r="H219" s="3"/>
       <c r="I219" s="3"/>
-      <c r="J219" s="8"/>
+      <c r="J219" s="7"/>
       <c r="K219" s="3"/>
       <c r="L219" s="3"/>
       <c r="M219" s="3"/>
@@ -8600,7 +8604,7 @@
       <c r="G220" s="3"/>
       <c r="H220" s="3"/>
       <c r="I220" s="3"/>
-      <c r="J220" s="8"/>
+      <c r="J220" s="7"/>
       <c r="K220" s="3"/>
       <c r="L220" s="3"/>
       <c r="M220" s="3"/>
@@ -8628,7 +8632,7 @@
       <c r="G221" s="3"/>
       <c r="H221" s="3"/>
       <c r="I221" s="3"/>
-      <c r="J221" s="8"/>
+      <c r="J221" s="7"/>
       <c r="K221" s="3"/>
       <c r="L221" s="3"/>
       <c r="M221" s="3"/>
@@ -8656,7 +8660,7 @@
       <c r="G222" s="3"/>
       <c r="H222" s="3"/>
       <c r="I222" s="3"/>
-      <c r="J222" s="8"/>
+      <c r="J222" s="7"/>
       <c r="K222" s="3"/>
       <c r="L222" s="3"/>
       <c r="M222" s="3"/>
@@ -8684,7 +8688,7 @@
       <c r="G223" s="3"/>
       <c r="H223" s="3"/>
       <c r="I223" s="3"/>
-      <c r="J223" s="8"/>
+      <c r="J223" s="7"/>
       <c r="K223" s="3"/>
       <c r="L223" s="3"/>
       <c r="M223" s="3"/>
@@ -8712,7 +8716,7 @@
       <c r="G224" s="3"/>
       <c r="H224" s="3"/>
       <c r="I224" s="3"/>
-      <c r="J224" s="8"/>
+      <c r="J224" s="7"/>
       <c r="K224" s="3"/>
       <c r="L224" s="3"/>
       <c r="M224" s="3"/>
@@ -8740,7 +8744,7 @@
       <c r="G225" s="3"/>
       <c r="H225" s="3"/>
       <c r="I225" s="3"/>
-      <c r="J225" s="8"/>
+      <c r="J225" s="7"/>
       <c r="K225" s="3"/>
       <c r="L225" s="3"/>
       <c r="M225" s="3"/>
@@ -8768,7 +8772,7 @@
       <c r="G226" s="3"/>
       <c r="H226" s="3"/>
       <c r="I226" s="3"/>
-      <c r="J226" s="8"/>
+      <c r="J226" s="7"/>
       <c r="K226" s="3"/>
       <c r="L226" s="3"/>
       <c r="M226" s="3"/>
@@ -8796,7 +8800,7 @@
       <c r="G227" s="3"/>
       <c r="H227" s="3"/>
       <c r="I227" s="3"/>
-      <c r="J227" s="8"/>
+      <c r="J227" s="7"/>
       <c r="K227" s="3"/>
       <c r="L227" s="3"/>
       <c r="M227" s="3"/>
@@ -8824,7 +8828,7 @@
       <c r="G228" s="3"/>
       <c r="H228" s="3"/>
       <c r="I228" s="3"/>
-      <c r="J228" s="8"/>
+      <c r="J228" s="7"/>
       <c r="K228" s="3"/>
       <c r="L228" s="3"/>
       <c r="M228" s="3"/>
@@ -9616,6 +9620,34 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:C22"/>
+    <mergeCell ref="D21:I22"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A25:C26"/>
+    <mergeCell ref="D25:F26"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="H14:I14"/>
     <mergeCell ref="A1:I10"/>
@@ -9625,37 +9657,9 @@
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A25:C26"/>
-    <mergeCell ref="D25:F26"/>
-    <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A21:C22"/>
-    <mergeCell ref="D21:I22"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D19" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D19" r:id="rId1"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>